<commit_message>
stm32 project setup and build
</commit_message>
<xml_diff>
--- a/02_Digital_HW_Design/Pin Assigments.xlsx
+++ b/02_Digital_HW_Design/Pin Assigments.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/skylar/Desktop/CAPSTONE/02_Digital_Design/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/skylar/Desktop/CAPSTONE/02_Digital_HW_Design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8960E632-C7A3-CD4F-8E62-D50E7B272620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6752B7F7-1F47-A24E-86A7-027635B7D2EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17700" xr2:uid="{FE3AA19E-76E0-5240-B00B-749D1CD90255}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="205">
   <si>
     <t>PROTO</t>
   </si>
@@ -50,15 +50,6 @@
     <t>DESC</t>
   </si>
   <si>
-    <t>I2C 1</t>
-  </si>
-  <si>
-    <t>I2C 2</t>
-  </si>
-  <si>
-    <t>I2C 3</t>
-  </si>
-  <si>
     <t>RESET</t>
   </si>
   <si>
@@ -239,9 +230,6 @@
     <t>PC9</t>
   </si>
   <si>
-    <t>I2C 4</t>
-  </si>
-  <si>
     <t>PC FN</t>
   </si>
   <si>
@@ -341,15 +329,6 @@
     <t>Sense if faders are being touched (from TTP223-BA6's output)</t>
   </si>
   <si>
-    <t>MCP23017 GPIO Expansion for encoders, buttons</t>
-  </si>
-  <si>
-    <t>MCP23017 GPIO Expansion for encoders, buttons + some CV DACs</t>
-  </si>
-  <si>
-    <t>Control Voltage DACs</t>
-  </si>
-  <si>
     <t>Fader1_ADC</t>
   </si>
   <si>
@@ -449,30 +428,6 @@
     <t>__MASTER_CS_in</t>
   </si>
   <si>
-    <t>Ctrl1_Clock</t>
-  </si>
-  <si>
-    <t>Ctrl1_Data</t>
-  </si>
-  <si>
-    <t>Ctrl2XCV_Clock</t>
-  </si>
-  <si>
-    <t>Ctrl2XCV_Data</t>
-  </si>
-  <si>
-    <t>CV1_Clock</t>
-  </si>
-  <si>
-    <t>CV1_Data</t>
-  </si>
-  <si>
-    <t>CV2_Clock</t>
-  </si>
-  <si>
-    <t>CV2_Data</t>
-  </si>
-  <si>
     <t>PC5</t>
   </si>
   <si>
@@ -657,6 +612,48 @@
   </si>
   <si>
     <t>PB6</t>
+  </si>
+  <si>
+    <t>MCP23017 GPIO Expansion x4, MCP4728 DAC x4</t>
+  </si>
+  <si>
+    <t>MCP23017 GPIO Expansion x8</t>
+  </si>
+  <si>
+    <t>I2C1_Clock</t>
+  </si>
+  <si>
+    <t>I2C1_Data</t>
+  </si>
+  <si>
+    <t>I2C2_Clock</t>
+  </si>
+  <si>
+    <t>I2C2_Data</t>
+  </si>
+  <si>
+    <t>I2C3_Clock</t>
+  </si>
+  <si>
+    <t>I2C3_Data</t>
+  </si>
+  <si>
+    <t>I2C4_Clock</t>
+  </si>
+  <si>
+    <t>I2C4_Data</t>
+  </si>
+  <si>
+    <t>I2C 1 400kHz</t>
+  </si>
+  <si>
+    <t>I2C 2 400kHz</t>
+  </si>
+  <si>
+    <t>I2C 3 400kHz</t>
+  </si>
+  <si>
+    <t>I2C 4 400kHz</t>
   </si>
 </sst>
 </file>
@@ -1060,61 +1057,61 @@
     <xf numFmtId="0" fontId="11" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1480,1221 +1477,1260 @@
         <v>0</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>68</v>
-      </c>
-      <c r="B2" s="56" t="s">
-        <v>100</v>
-      </c>
-      <c r="C2" s="56" t="s">
-        <v>3</v>
+      <c r="A2" s="48" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" s="48" t="s">
+        <v>191</v>
+      </c>
+      <c r="C2" s="48" t="s">
+        <v>201</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F2" s="9">
         <v>49</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>136</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" s="58"/>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
+      <c r="A3" s="49"/>
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
       <c r="D3" s="14" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F3" s="9">
         <v>50</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>137</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A4" s="59" t="s">
-        <v>80</v>
-      </c>
-      <c r="B4" s="59" t="s">
-        <v>101</v>
-      </c>
-      <c r="C4" s="59" t="s">
-        <v>4</v>
+      <c r="A4" s="50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4" s="50" t="s">
+        <v>191</v>
+      </c>
+      <c r="C4" s="50" t="s">
+        <v>202</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>182</v>
+        <v>167</v>
       </c>
       <c r="F4" s="20">
         <v>43</v>
       </c>
       <c r="G4" s="27" t="s">
-        <v>138</v>
+        <v>195</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A5" s="61"/>
-      <c r="B5" s="61"/>
-      <c r="C5" s="61"/>
+      <c r="A5" s="51"/>
+      <c r="B5" s="51"/>
+      <c r="C5" s="51"/>
       <c r="D5" s="26" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>183</v>
+        <v>168</v>
       </c>
       <c r="F5" s="20">
         <v>42</v>
       </c>
       <c r="G5" s="27" t="s">
-        <v>139</v>
+        <v>196</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A6" s="56" t="s">
-        <v>69</v>
-      </c>
-      <c r="B6" s="56" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6" s="56" t="s">
-        <v>5</v>
+      <c r="A6" s="48" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="48" t="s">
+        <v>191</v>
+      </c>
+      <c r="C6" s="48" t="s">
+        <v>203</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F6" s="9">
         <v>40</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>140</v>
+        <v>197</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A7" s="58"/>
-      <c r="B7" s="58"/>
-      <c r="C7" s="58"/>
+      <c r="A7" s="49"/>
+      <c r="B7" s="49"/>
+      <c r="C7" s="49"/>
       <c r="D7" s="14" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="F7" s="9">
         <v>58</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>141</v>
+        <v>198</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8" s="59" t="s">
-        <v>70</v>
-      </c>
-      <c r="B8" s="59" t="s">
-        <v>102</v>
-      </c>
-      <c r="C8" s="59" t="s">
+      <c r="A8" s="50" t="s">
         <v>66</v>
       </c>
+      <c r="B8" s="50" t="s">
+        <v>192</v>
+      </c>
+      <c r="C8" s="50" t="s">
+        <v>204</v>
+      </c>
       <c r="D8" s="26" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>196</v>
+        <v>181</v>
       </c>
       <c r="F8" s="20">
         <v>38</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>142</v>
+        <v>199</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9" s="61"/>
-      <c r="B9" s="61"/>
-      <c r="C9" s="61"/>
+      <c r="A9" s="51"/>
+      <c r="B9" s="51"/>
+      <c r="C9" s="51"/>
       <c r="D9" s="26" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>197</v>
+        <v>182</v>
       </c>
       <c r="F9" s="20">
         <v>39</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>143</v>
+        <v>200</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10" s="56" t="s">
-        <v>81</v>
+      <c r="A10" s="48" t="s">
+        <v>77</v>
       </c>
       <c r="B10" s="4"/>
-      <c r="C10" s="56" t="s">
+      <c r="C10" s="48" t="s">
+        <v>67</v>
+      </c>
+      <c r="D10" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="D10" s="14" t="s">
-        <v>75</v>
-      </c>
       <c r="E10" s="9" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F10" s="9">
         <v>19</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A11" s="57"/>
+      <c r="A11" s="58"/>
       <c r="B11" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="C11" s="57"/>
+        <v>83</v>
+      </c>
+      <c r="C11" s="58"/>
       <c r="D11" s="14" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="F11" s="9">
         <v>57</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A12" s="57"/>
+      <c r="A12" s="58"/>
       <c r="B12" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C12" s="57"/>
+        <v>78</v>
+      </c>
+      <c r="C12" s="58"/>
       <c r="D12" s="14" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F12" s="9">
         <v>21</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A13" s="58"/>
+      <c r="A13" s="49"/>
       <c r="B13" s="5"/>
-      <c r="C13" s="58"/>
+      <c r="C13" s="49"/>
       <c r="D13" s="14" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F13" s="9">
         <v>8</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="59" t="s">
-        <v>91</v>
+      <c r="A14" s="50" t="s">
+        <v>87</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>88</v>
-      </c>
-      <c r="C14" s="59" t="s">
-        <v>73</v>
+        <v>84</v>
+      </c>
+      <c r="C14" s="50" t="s">
+        <v>69</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F14" s="20">
         <v>35</v>
       </c>
       <c r="G14" s="21" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A15" s="60"/>
+      <c r="A15" s="57"/>
       <c r="B15" s="22" t="s">
-        <v>87</v>
-      </c>
-      <c r="C15" s="60"/>
+        <v>83</v>
+      </c>
+      <c r="C15" s="57"/>
       <c r="D15" s="19" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F15" s="20">
         <v>37</v>
       </c>
       <c r="G15" s="21" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A16" s="60"/>
+      <c r="A16" s="57"/>
       <c r="B16" s="22" t="s">
-        <v>85</v>
-      </c>
-      <c r="C16" s="60"/>
+        <v>81</v>
+      </c>
+      <c r="C16" s="57"/>
       <c r="D16" s="19" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="F16" s="20">
         <v>2</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="61"/>
+      <c r="A17" s="51"/>
       <c r="B17" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="C17" s="61"/>
+        <v>82</v>
+      </c>
+      <c r="C17" s="51"/>
       <c r="D17" s="19" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E17" s="20" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="F17" s="20">
         <v>11</v>
       </c>
       <c r="G17" s="21" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A18" s="56" t="s">
-        <v>92</v>
+      <c r="A18" s="48" t="s">
+        <v>88</v>
       </c>
       <c r="B18" s="25" t="s">
-        <v>88</v>
-      </c>
-      <c r="C18" s="56" t="s">
-        <v>72</v>
+        <v>84</v>
+      </c>
+      <c r="C18" s="48" t="s">
+        <v>68</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F18" s="9">
         <v>52</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A19" s="57"/>
+      <c r="A19" s="58"/>
       <c r="B19" s="25" t="s">
-        <v>87</v>
-      </c>
-      <c r="C19" s="57"/>
+        <v>83</v>
+      </c>
+      <c r="C19" s="58"/>
       <c r="D19" s="17" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F19" s="9">
         <v>54</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A20" s="57"/>
+      <c r="A20" s="58"/>
       <c r="B20" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="C20" s="57"/>
+        <v>78</v>
+      </c>
+      <c r="C20" s="58"/>
       <c r="D20" s="17" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="F20" s="9">
         <v>53</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A21" s="57"/>
+      <c r="A21" s="58"/>
       <c r="B21" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="C21" s="57"/>
+        <v>85</v>
+      </c>
+      <c r="C21" s="58"/>
       <c r="D21" s="17" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="F21" s="9">
         <v>59</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A22" s="58"/>
+      <c r="A22" s="49"/>
       <c r="B22" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="C22" s="58"/>
+        <v>86</v>
+      </c>
+      <c r="C22" s="49"/>
       <c r="D22" s="17" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F22" s="9">
         <v>60</v>
       </c>
       <c r="G22" s="14" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A23" s="49" t="s">
-        <v>93</v>
-      </c>
-      <c r="B23" s="49" t="s">
-        <v>25</v>
-      </c>
-      <c r="C23" s="49" t="s">
-        <v>95</v>
+      <c r="A23" s="52" t="s">
+        <v>89</v>
+      </c>
+      <c r="B23" s="52" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" s="52" t="s">
+        <v>91</v>
       </c>
       <c r="D23" s="26" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="E23" s="20" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F23" s="20">
         <v>12</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A24" s="49"/>
-      <c r="B24" s="49"/>
-      <c r="C24" s="49"/>
+      <c r="A24" s="52"/>
+      <c r="B24" s="52"/>
+      <c r="C24" s="52"/>
       <c r="D24" s="29" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="E24" s="20" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F24" s="20">
         <v>13</v>
       </c>
       <c r="G24" s="21" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A25" s="49"/>
-      <c r="B25" s="49"/>
-      <c r="C25" s="49"/>
+      <c r="A25" s="52"/>
+      <c r="B25" s="52"/>
+      <c r="C25" s="52"/>
       <c r="D25" s="29" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="E25" s="20" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F25" s="20">
         <v>14</v>
       </c>
       <c r="G25" s="21" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A26" s="49"/>
-      <c r="B26" s="49"/>
-      <c r="C26" s="49"/>
+      <c r="A26" s="52"/>
+      <c r="B26" s="52"/>
+      <c r="C26" s="52"/>
       <c r="D26" s="29" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="E26" s="20" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F26" s="20">
         <v>17</v>
       </c>
       <c r="G26" s="21" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A27" s="48" t="s">
-        <v>94</v>
-      </c>
-      <c r="B27" s="48" t="s">
-        <v>99</v>
-      </c>
-      <c r="C27" s="48" t="s">
-        <v>96</v>
+      <c r="A27" s="53" t="s">
+        <v>90</v>
+      </c>
+      <c r="B27" s="53" t="s">
+        <v>95</v>
+      </c>
+      <c r="C27" s="53" t="s">
+        <v>92</v>
       </c>
       <c r="D27" s="14"/>
       <c r="E27" s="9" t="s">
-        <v>191</v>
+        <v>176</v>
       </c>
       <c r="F27" s="9">
         <v>62</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A28" s="48"/>
-      <c r="B28" s="48"/>
-      <c r="C28" s="48"/>
+      <c r="A28" s="53"/>
+      <c r="B28" s="53"/>
+      <c r="C28" s="53"/>
       <c r="D28" s="14"/>
       <c r="E28" s="9" t="s">
-        <v>192</v>
+        <v>177</v>
       </c>
       <c r="F28" s="9">
         <v>55</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A29" s="48"/>
-      <c r="B29" s="48"/>
-      <c r="C29" s="48"/>
+      <c r="A29" s="53"/>
+      <c r="B29" s="53"/>
+      <c r="C29" s="53"/>
       <c r="D29" s="14"/>
       <c r="E29" s="9" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="F29" s="9">
         <v>25</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A30" s="48"/>
-      <c r="B30" s="48"/>
-      <c r="C30" s="48"/>
+      <c r="A30" s="53"/>
+      <c r="B30" s="53"/>
+      <c r="C30" s="53"/>
       <c r="D30" s="14"/>
       <c r="E30" s="9" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F30" s="9">
         <v>26</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="59" t="s">
-        <v>30</v>
-      </c>
-      <c r="B31" s="59" t="s">
-        <v>34</v>
-      </c>
-      <c r="C31" s="59" t="s">
-        <v>39</v>
-      </c>
-      <c r="D31" s="50" t="s">
-        <v>203</v>
+      <c r="A31" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="B31" s="50" t="s">
+        <v>31</v>
+      </c>
+      <c r="C31" s="50" t="s">
+        <v>36</v>
+      </c>
+      <c r="D31" s="59" t="s">
+        <v>188</v>
       </c>
       <c r="E31" s="20" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F31" s="20">
         <v>51</v>
       </c>
       <c r="G31" s="21" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A32" s="60"/>
-      <c r="B32" s="60"/>
-      <c r="C32" s="60"/>
-      <c r="D32" s="51"/>
+      <c r="A32" s="57"/>
+      <c r="B32" s="57"/>
+      <c r="C32" s="57"/>
+      <c r="D32" s="60"/>
       <c r="E32" s="20" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F32" s="20">
         <v>56</v>
       </c>
       <c r="G32" s="21" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A33" s="60"/>
-      <c r="B33" s="60"/>
-      <c r="C33" s="49" t="s">
-        <v>97</v>
-      </c>
-      <c r="D33" s="50" t="s">
-        <v>203</v>
+      <c r="A33" s="57"/>
+      <c r="B33" s="57"/>
+      <c r="C33" s="52" t="s">
+        <v>93</v>
+      </c>
+      <c r="D33" s="59" t="s">
+        <v>188</v>
       </c>
       <c r="E33" s="20" t="s">
-        <v>193</v>
+        <v>178</v>
       </c>
       <c r="F33" s="20">
         <v>30</v>
       </c>
       <c r="G33" s="21" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A34" s="60"/>
-      <c r="B34" s="60"/>
-      <c r="C34" s="49"/>
-      <c r="D34" s="51"/>
+      <c r="A34" s="57"/>
+      <c r="B34" s="57"/>
+      <c r="C34" s="52"/>
+      <c r="D34" s="60"/>
       <c r="E34" s="20" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="F34" s="20">
         <v>44</v>
       </c>
       <c r="G34" s="21" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="60"/>
-      <c r="B35" s="60"/>
-      <c r="C35" s="62" t="s">
-        <v>40</v>
-      </c>
-      <c r="D35" s="50" t="s">
-        <v>203</v>
+      <c r="A35" s="57"/>
+      <c r="B35" s="57"/>
+      <c r="C35" s="54" t="s">
+        <v>37</v>
+      </c>
+      <c r="D35" s="59" t="s">
+        <v>188</v>
       </c>
       <c r="E35" s="20" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F35" s="20">
         <v>20</v>
       </c>
       <c r="G35" s="21" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A36" s="60"/>
-      <c r="B36" s="60"/>
-      <c r="C36" s="63"/>
-      <c r="D36" s="51"/>
+      <c r="A36" s="57"/>
+      <c r="B36" s="57"/>
+      <c r="C36" s="55"/>
+      <c r="D36" s="60"/>
       <c r="E36" s="20" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F36" s="20">
         <v>18</v>
       </c>
       <c r="G36" s="21" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="60"/>
-      <c r="B37" s="60"/>
-      <c r="C37" s="64" t="s">
-        <v>98</v>
-      </c>
-      <c r="D37" s="50" t="s">
-        <v>203</v>
+      <c r="A37" s="57"/>
+      <c r="B37" s="57"/>
+      <c r="C37" s="56" t="s">
+        <v>94</v>
+      </c>
+      <c r="D37" s="59" t="s">
+        <v>188</v>
       </c>
       <c r="E37" s="20" t="s">
-        <v>195</v>
+        <v>180</v>
       </c>
       <c r="F37" s="20">
         <v>24</v>
       </c>
       <c r="G37" s="21" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A38" s="61"/>
-      <c r="B38" s="61"/>
-      <c r="C38" s="64"/>
-      <c r="D38" s="51"/>
+      <c r="A38" s="51"/>
+      <c r="B38" s="51"/>
+      <c r="C38" s="56"/>
+      <c r="D38" s="60"/>
       <c r="E38" s="20" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F38" s="20">
         <v>41</v>
       </c>
       <c r="G38" s="21" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A39" s="48" t="s">
-        <v>119</v>
-      </c>
-      <c r="B39" s="48" t="s">
-        <v>120</v>
-      </c>
-      <c r="C39" s="56" t="s">
-        <v>121</v>
+      <c r="A39" s="53" t="s">
+        <v>112</v>
+      </c>
+      <c r="B39" s="53" t="s">
+        <v>113</v>
+      </c>
+      <c r="C39" s="48" t="s">
+        <v>114</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F39" s="9">
         <v>34</v>
       </c>
       <c r="G39" s="7" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A40" s="48"/>
-      <c r="B40" s="48"/>
-      <c r="C40" s="57"/>
+      <c r="A40" s="53"/>
+      <c r="B40" s="53"/>
+      <c r="C40" s="58"/>
       <c r="D40" s="14" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F40" s="9">
         <v>33</v>
       </c>
       <c r="G40" s="7" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A41" s="48"/>
-      <c r="B41" s="48"/>
-      <c r="C41" s="58"/>
+      <c r="A41" s="53"/>
+      <c r="B41" s="53"/>
+      <c r="C41" s="49"/>
       <c r="D41" s="14" t="s">
-        <v>199</v>
+        <v>184</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F41" s="9">
         <v>36</v>
       </c>
       <c r="G41" s="7" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A42" s="48"/>
-      <c r="B42" s="48"/>
+      <c r="A42" s="53"/>
+      <c r="B42" s="53"/>
       <c r="C42" s="7" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F42" s="9">
         <v>9</v>
       </c>
       <c r="G42" s="7" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="21" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="B43" s="21" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="D43" s="21" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="E43" s="20" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F43" s="20">
         <v>10</v>
       </c>
       <c r="G43" s="28" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A44" s="54" t="s">
-        <v>153</v>
-      </c>
-      <c r="B44" s="54" t="s">
-        <v>154</v>
-      </c>
-      <c r="C44" s="54" t="s">
-        <v>155</v>
+      <c r="A44" s="61" t="s">
+        <v>138</v>
+      </c>
+      <c r="B44" s="61" t="s">
+        <v>139</v>
+      </c>
+      <c r="C44" s="61" t="s">
+        <v>140</v>
       </c>
       <c r="D44" s="30"/>
       <c r="E44" s="44" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F44" s="44">
         <v>5</v>
       </c>
       <c r="G44" s="31" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A45" s="55"/>
-      <c r="B45" s="55"/>
-      <c r="C45" s="55"/>
+      <c r="A45" s="62"/>
+      <c r="B45" s="62"/>
+      <c r="C45" s="62"/>
       <c r="D45" s="32"/>
       <c r="E45" s="45" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F45" s="45">
         <v>6</v>
       </c>
       <c r="G45" s="33" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A46" s="52" t="s">
-        <v>152</v>
-      </c>
-      <c r="B46" s="52" t="s">
-        <v>157</v>
-      </c>
-      <c r="C46" s="52" t="s">
-        <v>156</v>
+      <c r="A46" s="46" t="s">
+        <v>137</v>
+      </c>
+      <c r="B46" s="46" t="s">
+        <v>142</v>
+      </c>
+      <c r="C46" s="46" t="s">
+        <v>141</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
       <c r="E46" s="40" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F46" s="40">
         <v>46</v>
       </c>
       <c r="G46" s="34" t="s">
-        <v>158</v>
+        <v>143</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A47" s="53"/>
-      <c r="B47" s="53"/>
-      <c r="C47" s="53"/>
+      <c r="A47" s="47"/>
+      <c r="B47" s="47"/>
+      <c r="C47" s="47"/>
       <c r="D47" s="16" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="E47" s="40" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F47" s="40">
         <v>45</v>
       </c>
       <c r="G47" s="35" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A48" s="6" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="D48" s="15"/>
       <c r="E48" s="41" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F48" s="41">
         <v>7</v>
       </c>
       <c r="G48" s="11" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A49" s="52" t="s">
-        <v>8</v>
-      </c>
-      <c r="B49" s="52" t="s">
-        <v>145</v>
-      </c>
-      <c r="C49" s="52" t="s">
-        <v>7</v>
+      <c r="A49" s="46" t="s">
+        <v>5</v>
+      </c>
+      <c r="B49" s="46" t="s">
+        <v>130</v>
+      </c>
+      <c r="C49" s="46" t="s">
+        <v>4</v>
       </c>
       <c r="D49" s="16" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="E49" s="40" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F49" s="40">
         <v>22</v>
       </c>
       <c r="G49" s="10" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A50" s="53"/>
-      <c r="B50" s="53"/>
-      <c r="C50" s="53"/>
+      <c r="A50" s="47"/>
+      <c r="B50" s="47"/>
+      <c r="C50" s="47"/>
       <c r="D50" s="16" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="E50" s="40" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
       <c r="F50" s="40">
         <v>23</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="D51" s="15"/>
       <c r="E51" s="41" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F51" s="41">
         <v>27</v>
       </c>
       <c r="G51" s="11" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="8" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="D52" s="16"/>
       <c r="E52" s="40" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F52" s="40">
         <v>29</v>
       </c>
       <c r="G52" s="10" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="D53" s="15"/>
       <c r="E53" s="41" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F53" s="41">
         <v>1</v>
       </c>
       <c r="G53" s="11" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A54" s="8" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B54" s="8" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="D54" s="16"/>
       <c r="E54" s="40" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F54" s="40">
         <v>28</v>
       </c>
       <c r="G54" s="10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A55" s="48" t="s">
-        <v>165</v>
-      </c>
-      <c r="B55" s="48" t="s">
-        <v>166</v>
-      </c>
-      <c r="C55" s="48" t="s">
+      <c r="A55" s="53" t="s">
         <v>150</v>
+      </c>
+      <c r="B55" s="53" t="s">
+        <v>151</v>
+      </c>
+      <c r="C55" s="53" t="s">
+        <v>135</v>
       </c>
       <c r="D55" s="14"/>
       <c r="E55" s="41" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="F55" s="41">
         <v>16</v>
       </c>
       <c r="G55" s="11" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A56" s="48"/>
-      <c r="B56" s="48"/>
-      <c r="C56" s="48"/>
+      <c r="A56" s="53"/>
+      <c r="B56" s="53"/>
+      <c r="C56" s="53"/>
       <c r="D56" s="36"/>
       <c r="E56" s="41" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="F56" s="41">
         <v>32</v>
       </c>
       <c r="G56" s="11" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A57" s="48"/>
-      <c r="B57" s="48"/>
-      <c r="C57" s="48"/>
+      <c r="A57" s="53"/>
+      <c r="B57" s="53"/>
+      <c r="C57" s="53"/>
       <c r="D57" s="36"/>
       <c r="E57" s="41" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="F57" s="41">
         <v>48</v>
       </c>
       <c r="G57" s="11" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A58" s="48"/>
-      <c r="B58" s="48"/>
-      <c r="C58" s="48"/>
+      <c r="A58" s="53"/>
+      <c r="B58" s="53"/>
+      <c r="C58" s="53"/>
       <c r="D58" s="36"/>
       <c r="E58" s="41" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="F58" s="41">
         <v>64</v>
       </c>
       <c r="G58" s="11" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A59" s="49" t="s">
-        <v>168</v>
-      </c>
-      <c r="B59" s="49" t="s">
-        <v>167</v>
-      </c>
-      <c r="C59" s="49" t="s">
-        <v>150</v>
+      <c r="A59" s="52" t="s">
+        <v>153</v>
+      </c>
+      <c r="B59" s="52" t="s">
+        <v>152</v>
+      </c>
+      <c r="C59" s="52" t="s">
+        <v>135</v>
       </c>
       <c r="D59" s="26"/>
       <c r="E59" s="42" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="F59" s="42">
         <v>15</v>
       </c>
       <c r="G59" s="24" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A60" s="49"/>
-      <c r="B60" s="49"/>
-      <c r="C60" s="49"/>
+      <c r="A60" s="52"/>
+      <c r="B60" s="52"/>
+      <c r="C60" s="52"/>
       <c r="D60" s="26"/>
       <c r="E60" s="42" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="F60" s="42">
         <v>31</v>
       </c>
       <c r="G60" s="24" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A61" s="49"/>
-      <c r="B61" s="49"/>
-      <c r="C61" s="49"/>
+      <c r="A61" s="52"/>
+      <c r="B61" s="52"/>
+      <c r="C61" s="52"/>
       <c r="D61" s="26"/>
       <c r="E61" s="42" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="F61" s="42">
         <v>47</v>
       </c>
       <c r="G61" s="24" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A62" s="49"/>
-      <c r="B62" s="49"/>
-      <c r="C62" s="49"/>
+      <c r="A62" s="52"/>
+      <c r="B62" s="52"/>
+      <c r="C62" s="52"/>
       <c r="D62" s="26"/>
       <c r="E62" s="42" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="F62" s="42">
         <v>63</v>
       </c>
       <c r="G62" s="24" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
       <c r="C63" s="7"/>
       <c r="D63" s="7"/>
       <c r="E63" s="41" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F63" s="41">
         <v>61</v>
       </c>
       <c r="G63" s="37" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A64" s="63" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="64" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A64" s="46" t="s">
-        <v>184</v>
-      </c>
-      <c r="B64" s="46" t="s">
-        <v>185</v>
-      </c>
-      <c r="C64" s="46"/>
+      <c r="B64" s="63" t="s">
+        <v>170</v>
+      </c>
+      <c r="C64" s="63"/>
       <c r="D64" s="38"/>
       <c r="E64" s="43" t="s">
-        <v>186</v>
+        <v>171</v>
       </c>
       <c r="F64" s="43">
         <v>3</v>
       </c>
       <c r="G64" s="39" t="s">
-        <v>188</v>
+        <v>173</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A65" s="47"/>
-      <c r="B65" s="47"/>
-      <c r="C65" s="47"/>
+      <c r="A65" s="64"/>
+      <c r="B65" s="64"/>
+      <c r="C65" s="64"/>
       <c r="D65" s="38"/>
       <c r="E65" s="43" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="F65" s="43">
         <v>4</v>
       </c>
       <c r="G65" s="39" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="55">
+    <mergeCell ref="A64:A65"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="A55:A58"/>
+    <mergeCell ref="B55:B58"/>
+    <mergeCell ref="C55:C58"/>
+    <mergeCell ref="A59:A62"/>
+    <mergeCell ref="B59:B62"/>
+    <mergeCell ref="C59:C62"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="D37:D38"/>
+    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="A44:A45"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="C44:C45"/>
+    <mergeCell ref="A18:A22"/>
+    <mergeCell ref="C18:C22"/>
+    <mergeCell ref="A39:A42"/>
+    <mergeCell ref="B39:B42"/>
+    <mergeCell ref="C39:C41"/>
+    <mergeCell ref="B31:B38"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="C14:C17"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="C2:C3"/>
     <mergeCell ref="A49:A50"/>
     <mergeCell ref="C49:C50"/>
     <mergeCell ref="B49:B50"/>
@@ -2711,45 +2747,6 @@
     <mergeCell ref="C35:C36"/>
     <mergeCell ref="C37:C38"/>
     <mergeCell ref="A31:A38"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="C14:C17"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="A18:A22"/>
-    <mergeCell ref="C18:C22"/>
-    <mergeCell ref="A39:A42"/>
-    <mergeCell ref="B39:B42"/>
-    <mergeCell ref="C39:C41"/>
-    <mergeCell ref="B31:B38"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="D35:D36"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="D37:D38"/>
-    <mergeCell ref="A46:A47"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="A44:A45"/>
-    <mergeCell ref="B44:B45"/>
-    <mergeCell ref="C44:C45"/>
-    <mergeCell ref="A64:A65"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="C64:C65"/>
-    <mergeCell ref="A55:A58"/>
-    <mergeCell ref="B55:B58"/>
-    <mergeCell ref="C55:C58"/>
-    <mergeCell ref="A59:A62"/>
-    <mergeCell ref="B59:B62"/>
-    <mergeCell ref="C59:C62"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>